<commit_message>
Update README and classification scripts; enhance category taxonomy and outputs. Added `classify_full.py` for full classification, adjusted weights for phishing detection, and refined category labels in JSON files. Updated output files to reflect new classifications and improved reporting metrics.
</commit_message>
<xml_diff>
--- a/schemes/scheme2_balanced5/outputs/samples.xlsx
+++ b/schemes/scheme2_balanced5/outputs/samples.xlsx
@@ -824,12 +824,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>ac8pBTHVfL</t>
+          <t>l9g28bdfk0</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>AD 提前预订优惠政策年香港国际春季灯饰展 年香港国际春季灯饰展月日之前报名新客户折优惠老客户优惠年月日香港会议展览中心个参加春灯展的优胜之处一个全球参与的国际盛会产品齐备应有尽有现场推广活动提高宣传效益多项特别活动让您主动连系优质买家接触新兴市场买家抓紧商机提高对买家及媒体的曝光率优越的市中心位置一个全球参与的国际盛会年吸引来自个国家和地区超过家参展商年有来自个国家和地区逾名买家出席参 许贤松</t>
+          <t>Hi About of men in the country are dealing with ED as their health issue They are trying separate drug but only this one is assisting more than of them Try out this pill too and receive a private code...</t>
         </is>
       </c>
     </row>
@@ -847,12 +847,12 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>1xpgq8yHJ0</t>
+          <t>ac8pBTHVfL</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>不领双红包中的机会就失之交臂 您好不领双红包中的机会就失之交臂年双全球逛欢购物节来了点这里领取双红包每天都有机会领到以后在支付宝里面查看金额看手气和人品红包大小 [MONEY] [MONEY] [MONEY] [MONEY] [MONEY] 领用起止时间月日至月日红包使用时间月日至月日付定金立减进入数码家电预售会场祝您万事胜意 双</t>
+          <t>AD 提前预订优惠政策年香港国际春季灯饰展 年香港国际春季灯饰展月日之前报名新客户折优惠老客户优惠年月日香港会议展览中心个参加春灯展的优胜之处一个全球参与的国际盛会产品齐备应有尽有现场推广活动提高宣传效益多项特别活动让您主动连系优质买家接触新兴市场买家抓紧商机提高对买家及媒体的曝光率优越的市中心位置一个全球参与的国际盛会年吸引来自个国家和地区超过家参展商年有来自个国家和地区逾名买家出席参 许贤松</t>
         </is>
       </c>
     </row>
@@ -870,12 +870,12 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>MtgpR67bWv</t>
+          <t>1xpgq8yHJ0</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>get OFF on all products About of men in the world are dealing with Erectile Dysfunction as their health issue They are trying different medicine but only this one is helping more than of them Try out ...</t>
+          <t>不领双红包中的机会就失之交臂 您好不领双红包中的机会就失之交臂年双全球逛欢购物节来了点这里领取双红包每天都有机会领到以后在支付宝里面查看金额看手气和人品红包大小 [MONEY] [MONEY] [MONEY] [MONEY] [MONEY] 领用起止时间月日至月日红包使用时间月日至月日付定金立减进入数码家电预售会场祝您万事胜意 双</t>
         </is>
       </c>
     </row>
@@ -893,12 +893,12 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>fvlUaN6RWY</t>
+          <t>MtgpR67bWv</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Please add me on Linkedin networking let have good business deal Hi Hanson I d like to join your LinkedIn network [EMAIL] Hi [EMAIL] I d like to connect with you for immediate business transactions Am...</t>
+          <t>get OFF on all products About of men in the world are dealing with Erectile Dysfunction as their health issue They are trying different medicine but only this one is helping more than of them Try out ...</t>
         </is>
       </c>
     </row>
@@ -962,12 +962,12 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>x7bFmczNrE</t>
+          <t>w5GaOn13BS</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>人工智能 具体详情安排请查阅附件谢谢从网易邮箱发来的云附件人工智能复件 docx K 年月日到期在线预览下载 Python 深度学习</t>
+          <t>北京理工大学举办 EI index IOP ei 系列期刊出版 GSKI has been held successfully and have been indexed by E I And GSKI is sponsored by Chiang Mai University and Beijing Institute of Technology 本次会议将于年月日在广州召开这次会议将提供一个优...</t>
         </is>
       </c>
     </row>
@@ -985,12 +985,12 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>w5GaOn13BS</t>
+          <t>alm6kcpPy9</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>北京理工大学举办 EI index IOP ei 系列期刊出版 GSKI has been held successfully and have been indexed by E I And GSKI is sponsored by Chiang Mai University and Beijing Institute of Technology 本次会议将于年月日在广州召开这次会议将提供一个优...</t>
+          <t>SCI 投稿 SCI 发表首付免定金期刊正式录用后付款作者风险投稿网站立即查看 lunzi</t>
         </is>
       </c>
     </row>
@@ -1008,12 +1008,12 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>alm6kcpPy9</t>
+          <t>WBsqPbZy7g</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>SCI 投稿 SCI 发表首付免定金期刊正式录用后付款作者风险投稿网站立即查看 lunzi</t>
+          <t>关于科学前沿讲座的通知 同学您好第周年月日年月日人工智能学院开设科学前沿讲座安排如下讲座名称讲座人讲座时间讲座地点以用户为中心的社会多媒体计算徐常胜雁栖湖教一楼对抗生成网络及其应用研究赫然雁栖湖教一楼讲座及讲座人详细信息请留意海报内容或登录选课系统科学前沿讲座模块查看望同学们相互转告人工智能学院 [EMAIL]</t>
         </is>
       </c>
     </row>
@@ -1031,12 +1031,12 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>WBsqPbZy7g</t>
+          <t>iTlK2spqkE</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>关于科学前沿讲座的通知 同学您好第周年月日年月日人工智能学院开设科学前沿讲座安排如下讲座名称讲座人讲座时间讲座地点以用户为中心的社会多媒体计算徐常胜雁栖湖教一楼对抗生成网络及其应用研究赫然雁栖湖教一楼讲座及讲座人详细信息请留意海报内容或登录选课系统科学前沿讲座模块查看望同学们相互转告人工智能学院 [EMAIL]</t>
+          <t>学术交流您是我最永远的朋友 老师你好真诚致函敬请海涵我是北京育才文化的刘爱梅主打各刊物发表和专著出版欢迎您的咨询祝工作顺利咨询请加 [QQ] [WECHAT] bjhxtt 联系电话 [PHONE] 业务范围专著单书单号各学科均可指导写作并安排合适出版社出版国际会议 ISTP ISSHP CPCI S CPCI SSH 国际期刊 SCI A HCI SSCI 代写博士硕士论文中国教育报光明日报理论...</t>
         </is>
       </c>
     </row>
@@ -1054,12 +1054,12 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>iTlK2spqkE</t>
+          <t>FW0bUn1Ld3</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>学术交流您是我最永远的朋友 老师你好真诚致函敬请海涵我是北京育才文化的刘爱梅主打各刊物发表和专著出版欢迎您的咨询祝工作顺利咨询请加 [QQ] [WECHAT] bjhxtt 联系电话 [PHONE] 业务范围专著单书单号各学科均可指导写作并安排合适出版社出版国际会议 ISTP ISSHP CPCI S CPCI SSH 国际期刊 SCI A HCI SSCI 代写博士硕士论文中国教育报光明日报理论...</t>
+          <t>Invitation to The rd International Conference on Advanced Environmental Engineering 欢迎投稿 Welcome to ICAEE 第三届先进环境工程国际会议 ICAEE 第三届先进环境工程国际会议前正在筹备中欢迎投稿参会更多资讯请浏览会议网站 [URL] 来稿请投至 [EMAIL] 投稿时请在邮件主题中标明投稿字样并...</t>
         </is>
       </c>
     </row>
@@ -1077,12 +1077,12 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>FW0bUn1Ld3</t>
+          <t>p2j6LvcgT8</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Invitation to The rd International Conference on Advanced Environmental Engineering 欢迎投稿 Welcome to ICAEE 第三届先进环境工程国际会议 ICAEE 第三届先进环境工程国际会议前正在筹备中欢迎投稿参会更多资讯请浏览会议网站 [URL] 来稿请投至 [EMAIL] 投稿时请在邮件主题中标明投稿字样并...</t>
+          <t>Come to Guangzhou to witness CNAI IOP Journal of Physics for paper published Deadline Sincerely Invite Your Participation Welcome to the CNAI which will be held on December in Guangzhou China The nd s...</t>
         </is>
       </c>
     </row>
@@ -1100,12 +1100,12 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>p2j6LvcgT8</t>
+          <t>TOsDM3Fjni</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Come to Guangzhou to witness CNAI IOP Journal of Physics for paper published Deadline Sincerely Invite Your Participation Welcome to the CNAI which will be held on December in Guangzhou China The nd s...</t>
+          <t>We need your presence Dear Dr Sheng Xinzhi Greetings to you Based on your expertise we are pleased to welcome you at our nd Global Congress and Expo on Advancements of Laser Optics and Photonics confe...</t>
         </is>
       </c>
     </row>
@@ -1123,12 +1123,12 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>TOsDM3Fjni</t>
+          <t>HolePhbLzK</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>We need your presence Dear Dr Sheng Xinzhi Greetings to you Based on your expertise we are pleased to welcome you at our nd Global Congress and Expo on Advancements of Laser Optics and Photonics confe...</t>
+          <t>紧急约稿 SCI 加急 SCI 期刊录用后付款网站点击查看 guaixiuhw</t>
         </is>
       </c>
     </row>
@@ -1399,12 +1399,12 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>l9g28bdfk0</t>
+          <t>hkcifVzBAQ</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Hi About of men in the country are dealing with ED as their health issue They are trying separate drug but only this one is assisting more than of them Try out this pill too and receive a private code...</t>
+          <t>日报 appaPortal 日报 appaPortal 日报新版日报统计的范围包括 java sdk x cpp sdk DNA shell 其中平均调用时间统计范围 java sdk 消费的服务统计提供方服务名版本号请求次数响应次数成功次数响应成功率平均调用时间毫秒最多调用时间毫秒平均输入带宽字节最大输入带宽字节平均输出带宽字节最大输出带宽字节 GDNGdnCommonQuery GDNGdnM...</t>
         </is>
       </c>
     </row>
@@ -1422,12 +1422,12 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>hkcifVzBAQ</t>
+          <t>sajNtV1Awe</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>日报 appaPortal 日报 appaPortal 日报新版日报统计的范围包括 java sdk x cpp sdk DNA shell 其中平均调用时间统计范围 java sdk 消费的服务统计提供方服务名版本号请求次数响应次数成功次数响应成功率平均调用时间毫秒最多调用时间毫秒平均输入带宽字节最大输入带宽字节平均输出带宽字节最大输出带宽字节 GDNGdnCommonQuery GDNGdnM...</t>
+          <t>Rw libyang dlszgnubj</t>
         </is>
       </c>
     </row>
@@ -1445,12 +1445,12 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>sajNtV1Awe</t>
+          <t>Fi4HEJmYuU</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Rw libyang dlszgnubj</t>
+          <t>New Fatal Issue ImoNotifications java line imo stable [PHONE] imo stable Android [PHONE] com imo android imoim New Issue Just an FYI we detected a new fatal issue in ImoNotifications java line Learn m...</t>
         </is>
       </c>
     </row>
@@ -1468,12 +1468,12 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Fi4HEJmYuU</t>
+          <t>sA7Sz3Pqb4</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>New Fatal Issue ImoNotifications java line imo stable [PHONE] imo stable Android [PHONE] com imo android imoim New Issue Just an FYI we detected a new fatal issue in ImoNotifications java line Learn m...</t>
+          <t>northprod 用户复机错误 userId mmid xiaomi guonei 用户复机错误 [EMAIL]</t>
         </is>
       </c>
     </row>
@@ -1491,12 +1491,12 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>sA7Sz3Pqb4</t>
+          <t>HTaEtrUbhi</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>northprod 用户复机错误 userId mmid xiaomi guonei 用户复机错误 [EMAIL]</t>
+          <t>[PHONE] [EMAIL] [PHONE] ncncqwi</t>
         </is>
       </c>
     </row>
@@ -1514,12 +1514,12 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>VMCdHxhGeo</t>
+          <t>TOUt6E9CKF</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Tricks to help you this Halloween Tips and tricksto help the night go right Get spotted with Spotlight You can activate Spotlight and hold up your phone so your driver can spot your specific colored l...</t>
+          <t>New Fatal Issue d line imo beta [PHONE] imo beta Android [PHONE] com imo android imoimbeta New Issue Just an FYI we detected a new fatal issue in d line Learn more d line com fasterxml jackson core CD...</t>
         </is>
       </c>
     </row>
@@ -1537,12 +1537,12 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>oL5JpzGhaq</t>
+          <t>9pgfRPYZ8y</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Buongiorno Provaci [URL] Prenditi cura di te [EMAIL] giannico mario</t>
+          <t>frderjyxc</t>
         </is>
       </c>
     </row>
@@ -1560,12 +1560,12 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>cqGMR9J7l1</t>
+          <t>bDdnFRKj3f</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>您在 X MOL 的订阅邮件 亲爱的用户您选择的文献 Confining Hyperbranched Star Poly ethylene oxide Based Polymer into D Interpenetrating Network for High Performance All Solid State PolymerElectrolyte ACS Appl Mater Interfa...</t>
+          <t>玩 魏仕榕</t>
         </is>
       </c>
     </row>
@@ -1583,12 +1583,12 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>HTaEtrUbhi</t>
+          <t>auGpoi9EVl</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>[PHONE] [EMAIL] [PHONE] ncncqwi</t>
+          <t>aR e befcODRV V SZ</t>
         </is>
       </c>
     </row>
@@ -1736,12 +1736,12 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>iYRuZQ74zM</t>
+          <t>x7bFmczNrE</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>[EMAIL] 通知 您的邮箱长期未认证需要您及时登记备案否则将作离职处理禁止登陆登记地址 [URL] 服务支持 IT Serivce</t>
+          <t>人工智能 具体详情安排请查阅附件谢谢从网易邮箱发来的云附件人工智能复件 docx K 年月日到期在线预览下载 Python 深度学习</t>
         </is>
       </c>
     </row>
@@ -1759,12 +1759,12 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>oUgAzQBY9V</t>
+          <t>iYRuZQ74zM</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>SHIPMENT ETA NOTICE Hello sales Your shipment s listed below is scheduled for delivery tomorrow Tracking No Scheduled Delivery Date Tuesday October th Delivery Address Pending ValidationYou have the D...</t>
+          <t>[EMAIL] 通知 您的邮箱长期未认证需要您及时登记备案否则将作离职处理禁止登陆登记地址 [URL] 服务支持 IT Serivce</t>
         </is>
       </c>
     </row>
@@ -1782,12 +1782,12 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>w8fcL3npEi</t>
+          <t>oUgAzQBY9V</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>ATT URGENT [EMAIL] Someone sent you files via Wetransfer [EMAIL] Someone sent you files via Wetransfer items MB in total Will be deleted on November Hi [EMAIL] Based on our previous conversation I am ...</t>
+          <t>SHIPMENT ETA NOTICE Hello sales Your shipment s listed below is scheduled for delivery tomorrow Tracking No Scheduled Delivery Date Tuesday October th Delivery Address Pending ValidationYou have the D...</t>
         </is>
       </c>
     </row>
@@ -1805,12 +1805,12 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>yrvE95xFL4</t>
+          <t>w8fcL3npEi</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Liz [URL] Rosie Rosie Pack</t>
+          <t>ATT URGENT [EMAIL] Someone sent you files via Wetransfer [EMAIL] Someone sent you files via Wetransfer items MB in total Will be deleted on November Hi [EMAIL] Based on our previous conversation I am ...</t>
         </is>
       </c>
     </row>
@@ -1828,12 +1828,12 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>AuUjpNC6Eq</t>
+          <t>yrvE95xFL4</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Live Webinar Turn Away from Traditional Tethering and Towards a Better Method for Data Collection Turn Away from Traditional Tethering and Towards a Better Method for Data Collection Webinar Details T...</t>
+          <t>Liz [URL] Rosie Rosie Pack</t>
         </is>
       </c>
     </row>
@@ -1851,12 +1851,12 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>v1jfHVMS8O</t>
+          <t>AuUjpNC6Eq</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Florian [URL] Adam Adam Masterson</t>
+          <t>Live Webinar Turn Away from Traditional Tethering and Towards a Better Method for Data Collection Turn Away from Traditional Tethering and Towards a Better Method for Data Collection Webinar Details T...</t>
         </is>
       </c>
     </row>
@@ -1874,12 +1874,12 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>VIJGdiQor2</t>
+          <t>v1jfHVMS8O</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Tini [URL] koene wildschut koene wildschut</t>
+          <t>Florian [URL] Adam Adam Masterson</t>
         </is>
       </c>
     </row>
@@ -1897,12 +1897,12 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>lzSLNh6P9o</t>
+          <t>VIJGdiQor2</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>差点没把她搞虚脱 [URL] 差点没把她搞虚脱 neyad</t>
+          <t>Tini [URL] koene wildschut koene wildschut</t>
         </is>
       </c>
     </row>

</xml_diff>